<commit_message>
Rebuild every deliverable output with the seed data wording
All FRS, test plans, the register, the migration pack, the alignment pack and the process
deck are rebuilt so no retired wording remains in the Word, Excel and PowerPoint files.
Versions are kept (wording only). Two stale test plan references (BRD-1 message text,
BRD-5 volume 1 frontend test name) follow the current code. Drop indexes regenerated.
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/Migration/BIBS_Migration_BRD-13_Cutover_Task_Plan_v1.2.xlsx
+++ b/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/Migration/BIBS_Migration_BRD-13_Cutover_Task_Plan_v1.2.xlsx
@@ -4931,7 +4931,7 @@
       <c r="D16" s="12" t="inlineStr"/>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Legacy clean-up drives - UPP with no reference, invoices open more than 5 years, duplicate clients flagged in Mock 3, unmapped codes</t>
+          <t>Legacy clean-up drives - UPP with no reference, invoices open more than 5 years, duplicate clients flagged in Trial migration 3, unmapped codes</t>
         </is>
       </c>
       <c r="F16" s="12" t="inlineStr">
@@ -4945,7 +4945,7 @@
       <c r="H16" s="12" t="inlineStr"/>
       <c r="I16" s="12" t="inlineStr">
         <is>
-          <t>Clean-up tracker; counts reduced against Mock 3 profiling</t>
+          <t>Clean-up tracker; counts reduced against Trial migration 3 profiling</t>
         </is>
       </c>
       <c r="J16" s="12" t="inlineStr"/>
@@ -4977,7 +4977,7 @@
       <c r="D17" s="12" t="inlineStr"/>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Renewal processing team ready for the January expiries - staffing plan for January (handlers, overtime, back-up) signed; BIBS Renewal training completed; day-1 priority queue worked on the Mock 4 and dress-rehearsal data; draft RA-sent file from the Excel trackers validated and its rejects reviewed (maker-checker)</t>
+          <t>Renewal processing team ready for the January expiries - staffing plan for January (handlers, overtime, back-up) signed; BIBS Renewal training completed; day-1 priority queue worked on the Trial migration 4 and dress-rehearsal data; draft RA-sent file from the Excel trackers validated and its rejects reviewed (maker-checker)</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
@@ -5411,7 +5411,7 @@
       </c>
       <c r="I25" s="12" t="inlineStr">
         <is>
-          <t>Files CHECKED; counts against the Mock 4 volumes within 5 percent</t>
+          <t>Files CHECKED; counts against the Trial migration 4 volumes within 5 percent</t>
         </is>
       </c>
       <c r="J25" s="12" t="inlineStr"/>
@@ -11986,7 +11986,7 @@
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>Within 2 business days - root cause, new go-live date, which mocks to repeat; purge the production staging of the failed cutover within 5 days.</t>
+          <t>Within 2 business days - root cause, new go-live date, which trial migrations to repeat; purge the production staging of the failed cutover within 5 days.</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">

</xml_diff>